<commit_message>
Updated OPEX & EBITDA
</commit_message>
<xml_diff>
--- a/data/Сash_Flow_Budget.xlsx
+++ b/data/Сash_Flow_Budget.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22777" windowHeight="8665" tabRatio="924"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22777" windowHeight="8665" tabRatio="924" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Cash Flow Statement_Budget" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,11 @@
     <sheet name="Working Capital_Budget" sheetId="34" r:id="rId4"/>
     <sheet name="CapEx_Budget" sheetId="3" r:id="rId5"/>
     <sheet name="Debt Schedule_Budget" sheetId="6" r:id="rId6"/>
+    <sheet name="OPEX_Budget" sheetId="35" r:id="rId7"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId8"/>
+  </externalReferences>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="80">
   <si>
     <t>Indicator</t>
   </si>
@@ -219,6 +223,54 @@
   </si>
   <si>
     <t>Closing Loan Balance</t>
+  </si>
+  <si>
+    <t>OPEX Category</t>
+  </si>
+  <si>
+    <t>OPEX Subcategory</t>
+  </si>
+  <si>
+    <t>Salaries</t>
+  </si>
+  <si>
+    <t>Bonuses</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Internet &amp; Comunication</t>
+  </si>
+  <si>
+    <t>IT Servise</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Advertising</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Transportation</t>
+  </si>
+  <si>
+    <t>Business Trip</t>
+  </si>
+  <si>
+    <t>Environmental Cost</t>
+  </si>
+  <si>
+    <t>Write-offs</t>
+  </si>
+  <si>
+    <t>Taxes &amp; Fees</t>
+  </si>
+  <si>
+    <t>Health &amp; Safety</t>
   </si>
 </sst>
 </file>
@@ -952,6 +1004,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Cash Flow Statement_Actual"/>
+      <sheetName val="Sales_Actual"/>
+      <sheetName val="COGS_Actual"/>
+      <sheetName val="Working Capital_Actual"/>
+      <sheetName val="CapEx_Actual"/>
+      <sheetName val="Debt Schedule_Actual"/>
+      <sheetName val="DimDirection"/>
+      <sheetName val="OPEX_Actual"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="3">
+          <cell r="O3">
+            <v>0</v>
+          </cell>
+          <cell r="P3">
+            <v>0</v>
+          </cell>
+          <cell r="Q3">
+            <v>0</v>
+          </cell>
+          <cell r="R3">
+            <v>0</v>
+          </cell>
+          <cell r="S3">
+            <v>0</v>
+          </cell>
+          <cell r="T3">
+            <v>0</v>
+          </cell>
+          <cell r="U3">
+            <v>0</v>
+          </cell>
+          <cell r="V3">
+            <v>0</v>
+          </cell>
+          <cell r="W3">
+            <v>0</v>
+          </cell>
+          <cell r="X3">
+            <v>0</v>
+          </cell>
+          <cell r="Y3">
+            <v>0</v>
+          </cell>
+          <cell r="Z3">
+            <v>0</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2351,51 +2469,51 @@
       </c>
       <c r="C2" s="80">
         <f>B33</f>
-        <v>10270.216708271837</v>
+        <v>7024.2342646077959</v>
       </c>
       <c r="D2" s="80">
         <f t="shared" ref="D2:N2" si="0">C33</f>
-        <v>20264.948650358507</v>
+        <v>23701.584791462923</v>
       </c>
       <c r="E2" s="80">
         <f t="shared" si="0"/>
-        <v>47899.744650358494</v>
+        <v>60413.446894232242</v>
       </c>
       <c r="F2" s="80">
         <f t="shared" si="0"/>
-        <v>73477.780650358502</v>
+        <v>96025.370160270657</v>
       </c>
       <c r="G2" s="80">
         <f t="shared" si="0"/>
-        <v>17209.100650358501</v>
+        <v>47391.717559476587</v>
       </c>
       <c r="H2" s="80">
         <f t="shared" si="0"/>
-        <v>2590.7206503585039</v>
+        <v>44739.786835090999</v>
       </c>
       <c r="I2" s="80">
         <f t="shared" si="0"/>
-        <v>2379.9206503585083</v>
+        <v>56717.220066211004</v>
       </c>
       <c r="J2" s="80">
         <f t="shared" si="0"/>
-        <v>2491.5806503585118</v>
+        <v>72956.372642678994</v>
       </c>
       <c r="K2" s="80">
         <f t="shared" si="0"/>
-        <v>3519.5206503585141</v>
+        <v>89241.518571592838</v>
       </c>
       <c r="L2" s="80">
         <f t="shared" si="0"/>
-        <v>15810.360650358525</v>
+        <v>113720.17602304829</v>
       </c>
       <c r="M2" s="80">
         <f t="shared" si="0"/>
-        <v>21499.300650358527</v>
+        <v>139954.31670022113</v>
       </c>
       <c r="N2" s="80">
         <f t="shared" si="0"/>
-        <v>45050.520650358529</v>
+        <v>179505.96247004022</v>
       </c>
       <c r="O2" s="55">
         <v>0</v>
@@ -2834,43 +2952,43 @@
         <v>22</v>
       </c>
       <c r="B7" s="28">
-        <v>5000</v>
+        <v>5244.12</v>
       </c>
       <c r="C7" s="28">
-        <v>5000</v>
+        <v>5244.12</v>
       </c>
       <c r="D7" s="28">
-        <v>5000</v>
+        <v>5244.12</v>
       </c>
       <c r="E7" s="28">
-        <v>5000</v>
+        <v>5244.12</v>
       </c>
       <c r="F7" s="28">
-        <v>5000</v>
+        <v>5244.12</v>
       </c>
       <c r="G7" s="28">
-        <v>8000</v>
+        <v>6924.12</v>
       </c>
       <c r="H7" s="28">
-        <v>9000</v>
+        <v>6924.12</v>
       </c>
       <c r="I7" s="28">
-        <v>10000</v>
+        <v>6924.12</v>
       </c>
       <c r="J7" s="28">
-        <v>11000</v>
+        <v>6924.12</v>
       </c>
       <c r="K7" s="28">
-        <v>12000</v>
+        <v>8094.12</v>
       </c>
       <c r="L7" s="28">
-        <v>13000</v>
+        <v>8694.6721975362689</v>
       </c>
       <c r="M7" s="28">
-        <v>14000</v>
+        <v>8994.6721975362707</v>
       </c>
       <c r="N7" s="28">
-        <v>15000</v>
+        <v>9694.6721975362707</v>
       </c>
       <c r="O7" s="44">
         <v>0</v>
@@ -2914,43 +3032,43 @@
         <v>23</v>
       </c>
       <c r="B8" s="28">
-        <v>12860.004974020574</v>
+        <v>11574.400149220617</v>
       </c>
       <c r="C8" s="28">
-        <v>24447</v>
+        <v>21922.287496058001</v>
       </c>
       <c r="D8" s="28">
-        <v>30066</v>
+        <v>22154.108349416001</v>
       </c>
       <c r="E8" s="28">
-        <v>29205</v>
+        <v>18943.701752264002</v>
       </c>
       <c r="F8" s="28">
-        <v>24689</v>
+        <v>16837.417214879999</v>
       </c>
       <c r="G8" s="28">
-        <v>32470</v>
+        <v>26185.157345200001</v>
       </c>
       <c r="H8" s="28">
-        <v>31975</v>
+        <v>25276.290598799998</v>
       </c>
       <c r="I8" s="28">
-        <v>30938</v>
+        <v>20146.906013799999</v>
       </c>
       <c r="J8" s="28">
-        <v>20875</v>
+        <v>10927.390675085553</v>
       </c>
       <c r="K8" s="28">
-        <v>35783</v>
+        <v>29396.1415488536</v>
       </c>
       <c r="L8" s="28">
-        <v>43094</v>
+        <v>27733.603902001312</v>
       </c>
       <c r="M8" s="28">
-        <v>32551</v>
+        <v>21275.527714777978</v>
       </c>
       <c r="N8" s="28">
-        <v>32581</v>
+        <v>18191.177515200001</v>
       </c>
       <c r="O8" s="44">
         <v>0</v>
@@ -2994,43 +3112,43 @@
         <v>24</v>
       </c>
       <c r="B9" s="28">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="C9" s="28">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="D9" s="28">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E9" s="28">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="F9" s="28">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="G9" s="28">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="H9" s="28">
-        <v>20000</v>
+        <v>10100</v>
       </c>
       <c r="I9" s="28">
-        <v>20000</v>
+        <v>10100</v>
       </c>
       <c r="J9" s="28">
-        <v>20000</v>
+        <v>10200</v>
       </c>
       <c r="K9" s="28">
-        <v>20000</v>
+        <v>10200</v>
       </c>
       <c r="L9" s="28">
-        <v>20000</v>
+        <v>10200</v>
       </c>
       <c r="M9" s="28">
-        <v>20000</v>
+        <v>10300</v>
       </c>
       <c r="N9" s="28">
-        <v>20000</v>
+        <v>10300</v>
       </c>
       <c r="O9" s="44">
         <v>0</v>
@@ -3487,55 +3605,55 @@
       </c>
       <c r="B15" s="81">
         <f>B5+B6-B7-B8-B9-B10+B11-B12-B13+B14</f>
-        <v>10449.044766185165</v>
+        <v>6490.5295909851193</v>
       </c>
       <c r="C15" s="81">
         <f t="shared" ref="C15:N15" si="4">C5+C6-C7-C8-C9-C10+C11-C12-C13+C14</f>
-        <v>25458</v>
+        <v>32738.592503942004</v>
       </c>
       <c r="D15" s="81">
         <f t="shared" si="4"/>
-        <v>38069.799999999988</v>
+        <v>50737.571650583996</v>
       </c>
       <c r="E15" s="81">
         <f t="shared" si="4"/>
-        <v>38330</v>
+        <v>53347.17824773601</v>
       </c>
       <c r="F15" s="81">
         <f t="shared" si="4"/>
-        <v>33696</v>
+        <v>46303.462785120006</v>
       </c>
       <c r="G15" s="81">
         <f t="shared" si="4"/>
-        <v>50545</v>
+        <v>67905.722654800004</v>
       </c>
       <c r="H15" s="81">
         <f t="shared" si="4"/>
-        <v>43765</v>
+        <v>62439.589401200006</v>
       </c>
       <c r="I15" s="81">
         <f t="shared" si="4"/>
-        <v>47548</v>
+        <v>71314.973986199999</v>
       </c>
       <c r="J15" s="81">
         <f t="shared" si="4"/>
-        <v>16569</v>
+        <v>40392.489324914452</v>
       </c>
       <c r="K15" s="81">
         <f t="shared" si="4"/>
-        <v>75943</v>
+        <v>96035.738451146404</v>
       </c>
       <c r="L15" s="81">
         <f t="shared" si="4"/>
-        <v>58974</v>
+        <v>88439.723900462413</v>
       </c>
       <c r="M15" s="81">
         <f t="shared" si="4"/>
-        <v>40447</v>
+        <v>66427.800087685755</v>
       </c>
       <c r="N15" s="81">
         <f t="shared" si="4"/>
-        <v>74483</v>
+        <v>103878.15028726372</v>
       </c>
       <c r="O15" s="58">
         <f t="shared" ref="O15:Z15" si="5">O5+O6-O7-O8-O9+O11-O12-O13+O14</f>
@@ -3592,55 +3710,55 @@
       </c>
       <c r="B16" s="80">
         <f>B15*0.18</f>
-        <v>1880.8280579133295</v>
+        <v>1168.2953263773213</v>
       </c>
       <c r="C16" s="80">
         <f t="shared" ref="C16:N16" si="6">C15*0.18</f>
-        <v>4582.4399999999996</v>
+        <v>5892.9466507095603</v>
       </c>
       <c r="D16" s="80">
         <f t="shared" si="6"/>
-        <v>6852.5639999999976</v>
+        <v>9132.7628971051181</v>
       </c>
       <c r="E16" s="80">
         <f t="shared" si="6"/>
-        <v>6899.4</v>
+        <v>9602.4920845924808</v>
       </c>
       <c r="F16" s="80">
         <f t="shared" si="6"/>
-        <v>6065.28</v>
+        <v>8334.6233013216006</v>
       </c>
       <c r="G16" s="80">
         <f t="shared" si="6"/>
-        <v>9098.1</v>
+        <v>12223.030077863999</v>
       </c>
       <c r="H16" s="80">
         <f t="shared" si="6"/>
-        <v>7877.7</v>
+        <v>11239.126092216</v>
       </c>
       <c r="I16" s="80">
         <f t="shared" si="6"/>
-        <v>8558.64</v>
+        <v>12836.695317516</v>
       </c>
       <c r="J16" s="80">
         <f t="shared" si="6"/>
-        <v>2982.42</v>
+        <v>7270.6480784846008</v>
       </c>
       <c r="K16" s="80">
         <f t="shared" si="6"/>
-        <v>13669.74</v>
+        <v>17286.432921206353</v>
       </c>
       <c r="L16" s="80">
         <f t="shared" si="6"/>
-        <v>10615.32</v>
+        <v>15919.150302083233</v>
       </c>
       <c r="M16" s="80">
         <f t="shared" si="6"/>
-        <v>7280.46</v>
+        <v>11957.004015783436</v>
       </c>
       <c r="N16" s="80">
         <f t="shared" si="6"/>
-        <v>13406.939999999999</v>
+        <v>18698.067051707469</v>
       </c>
       <c r="O16" s="44">
         <f t="shared" ref="O16" si="7">O15*0.18</f>
@@ -3697,55 +3815,55 @@
       </c>
       <c r="B17" s="81">
         <f>B15-B16</f>
-        <v>8568.2167082718352</v>
+        <v>5322.2342646077977</v>
       </c>
       <c r="C17" s="81">
         <f t="shared" ref="C17:N17" si="9">C15-C16</f>
-        <v>20875.560000000001</v>
+        <v>26845.645853232443</v>
       </c>
       <c r="D17" s="81">
         <f t="shared" si="9"/>
-        <v>31217.23599999999</v>
+        <v>41604.808753478879</v>
       </c>
       <c r="E17" s="81">
         <f t="shared" si="9"/>
-        <v>31430.6</v>
+        <v>43744.686163143531</v>
       </c>
       <c r="F17" s="81">
         <f t="shared" si="9"/>
-        <v>27630.720000000001</v>
+        <v>37968.839483798409</v>
       </c>
       <c r="G17" s="81">
         <f t="shared" si="9"/>
-        <v>41446.9</v>
+        <v>55682.692576936002</v>
       </c>
       <c r="H17" s="81">
         <f t="shared" si="9"/>
-        <v>35887.300000000003</v>
+        <v>51200.463308984006</v>
       </c>
       <c r="I17" s="81">
         <f t="shared" si="9"/>
-        <v>38989.360000000001</v>
+        <v>58478.278668683997</v>
       </c>
       <c r="J17" s="81">
         <f t="shared" si="9"/>
-        <v>13586.58</v>
+        <v>33121.841246429853</v>
       </c>
       <c r="K17" s="81">
         <f t="shared" si="9"/>
-        <v>62273.26</v>
+        <v>78749.305529940058</v>
       </c>
       <c r="L17" s="81">
         <f t="shared" si="9"/>
-        <v>48358.68</v>
+        <v>72520.573598379182</v>
       </c>
       <c r="M17" s="81">
         <f t="shared" si="9"/>
-        <v>33166.54</v>
+        <v>54470.796071902318</v>
       </c>
       <c r="N17" s="81">
         <f t="shared" si="9"/>
-        <v>61076.06</v>
+        <v>85180.08323555626</v>
       </c>
       <c r="O17" s="58">
         <f t="shared" ref="O17" si="10">O15-O16</f>
@@ -4097,55 +4215,55 @@
       </c>
       <c r="B21" s="84">
         <f>B17+B10-B18-B19+B20-3520</f>
-        <v>16270.216708271837</v>
+        <v>13024.234264607796</v>
       </c>
       <c r="C21" s="84">
         <f>C17+C10-C18-C19+C20-B16</f>
-        <v>23994.73194208667</v>
+        <v>30677.350526855127</v>
       </c>
       <c r="D21" s="84">
         <f t="shared" ref="D21:N21" si="12">D17+D10-D18-D19+D20-C16</f>
-        <v>41634.795999999988</v>
+        <v>50711.862102769315</v>
       </c>
       <c r="E21" s="84">
         <f t="shared" si="12"/>
-        <v>39578.036</v>
+        <v>49611.923266038415</v>
       </c>
       <c r="F21" s="84">
         <f t="shared" si="12"/>
-        <v>-4268.6799999999985</v>
+        <v>3366.347399205928</v>
       </c>
       <c r="G21" s="84">
         <f t="shared" si="12"/>
-        <v>30381.620000000003</v>
+        <v>42348.069275614413</v>
       </c>
       <c r="H21" s="84">
         <f t="shared" si="12"/>
-        <v>41789.200000000004</v>
+        <v>53977.433231120005</v>
       </c>
       <c r="I21" s="84">
         <f t="shared" si="12"/>
-        <v>16111.66</v>
+        <v>32239.152576467997</v>
       </c>
       <c r="J21" s="84">
         <f t="shared" si="12"/>
-        <v>20027.940000000002</v>
+        <v>35285.145928913851</v>
       </c>
       <c r="K21" s="84">
         <f t="shared" si="12"/>
-        <v>74290.840000000011</v>
+        <v>86478.657451455452</v>
       </c>
       <c r="L21" s="84">
         <f t="shared" si="12"/>
-        <v>19688.940000000002</v>
+        <v>40234.140677172829</v>
       </c>
       <c r="M21" s="84">
         <f t="shared" si="12"/>
-        <v>37551.22</v>
+        <v>53551.645769819093</v>
       </c>
       <c r="N21" s="84">
         <f t="shared" si="12"/>
-        <v>28795.599999999999</v>
+        <v>48223.079219772822</v>
       </c>
       <c r="O21" s="84">
         <v>0</v>
@@ -5114,55 +5232,55 @@
       </c>
       <c r="B32" s="84">
         <f>B21+B23+B31</f>
-        <v>2270.216708271837</v>
+        <v>-975.76573539220408</v>
       </c>
       <c r="C32" s="84">
         <f t="shared" ref="C32:F32" si="19">C21+C23+C31</f>
-        <v>9994.7319420866697</v>
+        <v>16677.350526855127</v>
       </c>
       <c r="D32" s="84">
         <f t="shared" si="19"/>
-        <v>27634.795999999988</v>
+        <v>36711.862102769315</v>
       </c>
       <c r="E32" s="84">
         <f t="shared" si="19"/>
-        <v>25578.036</v>
+        <v>35611.923266038415</v>
       </c>
       <c r="F32" s="84">
         <f t="shared" si="19"/>
-        <v>-56268.68</v>
+        <v>-48633.65260079407</v>
       </c>
       <c r="G32" s="84">
         <f>G21+G23+G31</f>
-        <v>-14618.379999999997</v>
+        <v>-2651.9307243855874</v>
       </c>
       <c r="H32" s="84">
         <f t="shared" ref="H32:O32" si="20">H21+H23+H31</f>
-        <v>-210.79999999999563</v>
+        <v>11977.433231120005</v>
       </c>
       <c r="I32" s="84">
         <f t="shared" si="20"/>
-        <v>111.66000000000349</v>
+        <v>16239.152576467997</v>
       </c>
       <c r="J32" s="84">
         <f t="shared" si="20"/>
-        <v>1027.9400000000023</v>
+        <v>16285.145928913851</v>
       </c>
       <c r="K32" s="84">
         <f t="shared" si="20"/>
-        <v>12290.840000000011</v>
+        <v>24478.657451455452</v>
       </c>
       <c r="L32" s="84">
         <f t="shared" si="20"/>
-        <v>5688.9400000000023</v>
+        <v>26234.140677172829</v>
       </c>
       <c r="M32" s="84">
         <f t="shared" si="20"/>
-        <v>23551.22</v>
+        <v>39551.645769819093</v>
       </c>
       <c r="N32" s="84">
         <f t="shared" si="20"/>
-        <v>14795.599999999999</v>
+        <v>34223.079219772822</v>
       </c>
       <c r="O32" s="59">
         <f t="shared" si="20"/>
@@ -5219,55 +5337,55 @@
       </c>
       <c r="B33" s="87">
         <f t="shared" ref="B33:Z33" si="22">B32+B2</f>
-        <v>10270.216708271837</v>
+        <v>7024.2342646077959</v>
       </c>
       <c r="C33" s="87">
         <f t="shared" si="22"/>
-        <v>20264.948650358507</v>
+        <v>23701.584791462923</v>
       </c>
       <c r="D33" s="87">
         <f t="shared" si="22"/>
-        <v>47899.744650358494</v>
+        <v>60413.446894232242</v>
       </c>
       <c r="E33" s="87">
         <f t="shared" si="22"/>
-        <v>73477.780650358502</v>
+        <v>96025.370160270657</v>
       </c>
       <c r="F33" s="87">
         <f t="shared" si="22"/>
-        <v>17209.100650358501</v>
+        <v>47391.717559476587</v>
       </c>
       <c r="G33" s="87">
         <f t="shared" si="22"/>
-        <v>2590.7206503585039</v>
+        <v>44739.786835090999</v>
       </c>
       <c r="H33" s="87">
         <f t="shared" si="22"/>
-        <v>2379.9206503585083</v>
+        <v>56717.220066211004</v>
       </c>
       <c r="I33" s="87">
         <f t="shared" si="22"/>
-        <v>2491.5806503585118</v>
+        <v>72956.372642678994</v>
       </c>
       <c r="J33" s="87">
         <f t="shared" si="22"/>
-        <v>3519.5206503585141</v>
+        <v>89241.518571592838</v>
       </c>
       <c r="K33" s="87">
         <f t="shared" si="22"/>
-        <v>15810.360650358525</v>
+        <v>113720.17602304829</v>
       </c>
       <c r="L33" s="87">
         <f t="shared" si="22"/>
-        <v>21499.300650358527</v>
+        <v>139954.31670022113</v>
       </c>
       <c r="M33" s="87">
         <f t="shared" si="22"/>
-        <v>45050.520650358529</v>
+        <v>179505.96247004022</v>
       </c>
       <c r="N33" s="87">
         <f t="shared" si="22"/>
-        <v>59846.120650358527</v>
+        <v>213729.04168981305</v>
       </c>
       <c r="O33" s="59">
         <f t="shared" si="22"/>
@@ -16345,4 +16463,2679 @@
   <pageMargins left="0.26" right="0.70866141732283472" top="0.28999999999999998" bottom="0.2" header="0.2" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AA17"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="11.3" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="38.109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" style="13" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" style="13" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="14" style="13" customWidth="1"/>
+    <col min="9" max="9" width="12" style="13" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" style="13" customWidth="1"/>
+    <col min="11" max="11" width="13" style="13" customWidth="1"/>
+    <col min="12" max="12" width="14" style="13" customWidth="1"/>
+    <col min="13" max="13" width="12" style="13" customWidth="1"/>
+    <col min="14" max="14" width="10" style="13" customWidth="1"/>
+    <col min="15" max="15" width="13" style="13" customWidth="1"/>
+    <col min="16" max="16" width="14" style="13" customWidth="1"/>
+    <col min="17" max="17" width="12" style="13" customWidth="1"/>
+    <col min="18" max="18" width="10" style="13" customWidth="1"/>
+    <col min="19" max="19" width="13" style="13" customWidth="1"/>
+    <col min="20" max="20" width="14" style="13" customWidth="1"/>
+    <col min="21" max="21" width="12" style="13" customWidth="1"/>
+    <col min="22" max="22" width="10" style="13" customWidth="1"/>
+    <col min="23" max="23" width="13" style="13" customWidth="1"/>
+    <col min="24" max="24" width="14" style="13" customWidth="1"/>
+    <col min="25" max="25" width="12" style="13" customWidth="1"/>
+    <col min="26" max="26" width="10" style="13" customWidth="1"/>
+    <col min="27" max="27" width="13" style="13" customWidth="1"/>
+    <col min="28" max="224" width="8.88671875" style="13"/>
+    <col min="225" max="225" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="226" max="226" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="227" max="227" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="228" max="228" width="10" style="13" customWidth="1"/>
+    <col min="229" max="229" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="230" max="230" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="231" max="231" width="13.44140625" style="13" customWidth="1"/>
+    <col min="232" max="232" width="12.109375" style="13" customWidth="1"/>
+    <col min="233" max="233" width="11.88671875" style="13" customWidth="1"/>
+    <col min="234" max="234" width="12.44140625" style="13" customWidth="1"/>
+    <col min="235" max="235" width="11.44140625" style="13" customWidth="1"/>
+    <col min="236" max="236" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="237" max="237" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="238" max="238" width="11.44140625" style="13" customWidth="1"/>
+    <col min="239" max="239" width="9.109375" style="13" customWidth="1"/>
+    <col min="240" max="241" width="10" style="13" customWidth="1"/>
+    <col min="242" max="242" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="243" max="480" width="8.88671875" style="13"/>
+    <col min="481" max="481" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="482" max="482" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="483" max="483" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="484" max="484" width="10" style="13" customWidth="1"/>
+    <col min="485" max="485" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="486" max="486" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="487" max="487" width="13.44140625" style="13" customWidth="1"/>
+    <col min="488" max="488" width="12.109375" style="13" customWidth="1"/>
+    <col min="489" max="489" width="11.88671875" style="13" customWidth="1"/>
+    <col min="490" max="490" width="12.44140625" style="13" customWidth="1"/>
+    <col min="491" max="491" width="11.44140625" style="13" customWidth="1"/>
+    <col min="492" max="492" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="493" max="493" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="494" max="494" width="11.44140625" style="13" customWidth="1"/>
+    <col min="495" max="495" width="9.109375" style="13" customWidth="1"/>
+    <col min="496" max="497" width="10" style="13" customWidth="1"/>
+    <col min="498" max="498" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="499" max="736" width="8.88671875" style="13"/>
+    <col min="737" max="737" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="738" max="738" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="739" max="739" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="740" max="740" width="10" style="13" customWidth="1"/>
+    <col min="741" max="741" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="742" max="742" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="743" max="743" width="13.44140625" style="13" customWidth="1"/>
+    <col min="744" max="744" width="12.109375" style="13" customWidth="1"/>
+    <col min="745" max="745" width="11.88671875" style="13" customWidth="1"/>
+    <col min="746" max="746" width="12.44140625" style="13" customWidth="1"/>
+    <col min="747" max="747" width="11.44140625" style="13" customWidth="1"/>
+    <col min="748" max="748" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="749" max="749" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="750" max="750" width="11.44140625" style="13" customWidth="1"/>
+    <col min="751" max="751" width="9.109375" style="13" customWidth="1"/>
+    <col min="752" max="753" width="10" style="13" customWidth="1"/>
+    <col min="754" max="754" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="755" max="992" width="8.88671875" style="13"/>
+    <col min="993" max="993" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="994" max="994" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="995" max="995" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="996" max="996" width="10" style="13" customWidth="1"/>
+    <col min="997" max="997" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="998" max="998" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="999" max="999" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1000" max="1000" width="12.109375" style="13" customWidth="1"/>
+    <col min="1001" max="1001" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1002" max="1002" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1003" max="1003" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1004" max="1004" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1005" max="1005" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1006" max="1006" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1007" max="1007" width="9.109375" style="13" customWidth="1"/>
+    <col min="1008" max="1009" width="10" style="13" customWidth="1"/>
+    <col min="1010" max="1010" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1011" max="1248" width="8.88671875" style="13"/>
+    <col min="1249" max="1249" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1250" max="1250" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1251" max="1251" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1252" max="1252" width="10" style="13" customWidth="1"/>
+    <col min="1253" max="1253" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1254" max="1254" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1255" max="1255" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1256" max="1256" width="12.109375" style="13" customWidth="1"/>
+    <col min="1257" max="1257" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1258" max="1258" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1259" max="1259" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1260" max="1260" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1261" max="1261" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1262" max="1262" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1263" max="1263" width="9.109375" style="13" customWidth="1"/>
+    <col min="1264" max="1265" width="10" style="13" customWidth="1"/>
+    <col min="1266" max="1266" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1267" max="1504" width="8.88671875" style="13"/>
+    <col min="1505" max="1505" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1506" max="1506" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1507" max="1507" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1508" max="1508" width="10" style="13" customWidth="1"/>
+    <col min="1509" max="1509" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1510" max="1510" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1511" max="1511" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1512" max="1512" width="12.109375" style="13" customWidth="1"/>
+    <col min="1513" max="1513" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1514" max="1514" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1515" max="1515" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1516" max="1516" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1517" max="1517" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1518" max="1518" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1519" max="1519" width="9.109375" style="13" customWidth="1"/>
+    <col min="1520" max="1521" width="10" style="13" customWidth="1"/>
+    <col min="1522" max="1522" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1523" max="1760" width="8.88671875" style="13"/>
+    <col min="1761" max="1761" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1762" max="1762" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1763" max="1763" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1764" max="1764" width="10" style="13" customWidth="1"/>
+    <col min="1765" max="1765" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1766" max="1766" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1767" max="1767" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1768" max="1768" width="12.109375" style="13" customWidth="1"/>
+    <col min="1769" max="1769" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1770" max="1770" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1771" max="1771" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1772" max="1772" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1773" max="1773" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1774" max="1774" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1775" max="1775" width="9.109375" style="13" customWidth="1"/>
+    <col min="1776" max="1777" width="10" style="13" customWidth="1"/>
+    <col min="1778" max="1778" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1779" max="2016" width="8.88671875" style="13"/>
+    <col min="2017" max="2017" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2018" max="2018" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2019" max="2019" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2020" max="2020" width="10" style="13" customWidth="1"/>
+    <col min="2021" max="2021" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2022" max="2022" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2023" max="2023" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2024" max="2024" width="12.109375" style="13" customWidth="1"/>
+    <col min="2025" max="2025" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2026" max="2026" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2027" max="2027" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2028" max="2028" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2029" max="2029" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2030" max="2030" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2031" max="2031" width="9.109375" style="13" customWidth="1"/>
+    <col min="2032" max="2033" width="10" style="13" customWidth="1"/>
+    <col min="2034" max="2034" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2035" max="2272" width="8.88671875" style="13"/>
+    <col min="2273" max="2273" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2274" max="2274" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2275" max="2275" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2276" max="2276" width="10" style="13" customWidth="1"/>
+    <col min="2277" max="2277" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2278" max="2278" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2279" max="2279" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2280" max="2280" width="12.109375" style="13" customWidth="1"/>
+    <col min="2281" max="2281" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2282" max="2282" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2283" max="2283" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2284" max="2284" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2285" max="2285" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2286" max="2286" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2287" max="2287" width="9.109375" style="13" customWidth="1"/>
+    <col min="2288" max="2289" width="10" style="13" customWidth="1"/>
+    <col min="2290" max="2290" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2291" max="2528" width="8.88671875" style="13"/>
+    <col min="2529" max="2529" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2530" max="2530" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2531" max="2531" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2532" max="2532" width="10" style="13" customWidth="1"/>
+    <col min="2533" max="2533" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2534" max="2534" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2535" max="2535" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2536" max="2536" width="12.109375" style="13" customWidth="1"/>
+    <col min="2537" max="2537" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2538" max="2538" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2539" max="2539" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2540" max="2540" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2541" max="2541" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2542" max="2542" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2543" max="2543" width="9.109375" style="13" customWidth="1"/>
+    <col min="2544" max="2545" width="10" style="13" customWidth="1"/>
+    <col min="2546" max="2546" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2547" max="2784" width="8.88671875" style="13"/>
+    <col min="2785" max="2785" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2786" max="2786" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2787" max="2787" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2788" max="2788" width="10" style="13" customWidth="1"/>
+    <col min="2789" max="2789" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2790" max="2790" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2791" max="2791" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2792" max="2792" width="12.109375" style="13" customWidth="1"/>
+    <col min="2793" max="2793" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2794" max="2794" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2795" max="2795" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2796" max="2796" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2797" max="2797" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2798" max="2798" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2799" max="2799" width="9.109375" style="13" customWidth="1"/>
+    <col min="2800" max="2801" width="10" style="13" customWidth="1"/>
+    <col min="2802" max="2802" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2803" max="3040" width="8.88671875" style="13"/>
+    <col min="3041" max="3041" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3042" max="3042" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3043" max="3043" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3044" max="3044" width="10" style="13" customWidth="1"/>
+    <col min="3045" max="3045" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3046" max="3046" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3047" max="3047" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3048" max="3048" width="12.109375" style="13" customWidth="1"/>
+    <col min="3049" max="3049" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3050" max="3050" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3051" max="3051" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3052" max="3052" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3053" max="3053" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3054" max="3054" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3055" max="3055" width="9.109375" style="13" customWidth="1"/>
+    <col min="3056" max="3057" width="10" style="13" customWidth="1"/>
+    <col min="3058" max="3058" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3059" max="3296" width="8.88671875" style="13"/>
+    <col min="3297" max="3297" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3298" max="3298" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3299" max="3299" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3300" max="3300" width="10" style="13" customWidth="1"/>
+    <col min="3301" max="3301" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3302" max="3302" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3303" max="3303" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3304" max="3304" width="12.109375" style="13" customWidth="1"/>
+    <col min="3305" max="3305" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3306" max="3306" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3307" max="3307" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3308" max="3308" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3309" max="3309" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3310" max="3310" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3311" max="3311" width="9.109375" style="13" customWidth="1"/>
+    <col min="3312" max="3313" width="10" style="13" customWidth="1"/>
+    <col min="3314" max="3314" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3315" max="3552" width="8.88671875" style="13"/>
+    <col min="3553" max="3553" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3554" max="3554" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3555" max="3555" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3556" max="3556" width="10" style="13" customWidth="1"/>
+    <col min="3557" max="3557" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3558" max="3558" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3559" max="3559" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3560" max="3560" width="12.109375" style="13" customWidth="1"/>
+    <col min="3561" max="3561" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3562" max="3562" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3563" max="3563" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3564" max="3564" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3565" max="3565" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3566" max="3566" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3567" max="3567" width="9.109375" style="13" customWidth="1"/>
+    <col min="3568" max="3569" width="10" style="13" customWidth="1"/>
+    <col min="3570" max="3570" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3571" max="3808" width="8.88671875" style="13"/>
+    <col min="3809" max="3809" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3810" max="3810" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3811" max="3811" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3812" max="3812" width="10" style="13" customWidth="1"/>
+    <col min="3813" max="3813" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3814" max="3814" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3815" max="3815" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3816" max="3816" width="12.109375" style="13" customWidth="1"/>
+    <col min="3817" max="3817" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3818" max="3818" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3819" max="3819" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3820" max="3820" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3821" max="3821" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3822" max="3822" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3823" max="3823" width="9.109375" style="13" customWidth="1"/>
+    <col min="3824" max="3825" width="10" style="13" customWidth="1"/>
+    <col min="3826" max="3826" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3827" max="4064" width="8.88671875" style="13"/>
+    <col min="4065" max="4065" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4066" max="4066" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4067" max="4067" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4068" max="4068" width="10" style="13" customWidth="1"/>
+    <col min="4069" max="4069" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4070" max="4070" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4071" max="4071" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4072" max="4072" width="12.109375" style="13" customWidth="1"/>
+    <col min="4073" max="4073" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4074" max="4074" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4075" max="4075" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4076" max="4076" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4077" max="4077" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4078" max="4078" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4079" max="4079" width="9.109375" style="13" customWidth="1"/>
+    <col min="4080" max="4081" width="10" style="13" customWidth="1"/>
+    <col min="4082" max="4082" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4083" max="4320" width="8.88671875" style="13"/>
+    <col min="4321" max="4321" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4322" max="4322" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4323" max="4323" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4324" max="4324" width="10" style="13" customWidth="1"/>
+    <col min="4325" max="4325" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4326" max="4326" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4327" max="4327" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4328" max="4328" width="12.109375" style="13" customWidth="1"/>
+    <col min="4329" max="4329" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4330" max="4330" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4331" max="4331" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4332" max="4332" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4333" max="4333" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4334" max="4334" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4335" max="4335" width="9.109375" style="13" customWidth="1"/>
+    <col min="4336" max="4337" width="10" style="13" customWidth="1"/>
+    <col min="4338" max="4338" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4339" max="4576" width="8.88671875" style="13"/>
+    <col min="4577" max="4577" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4578" max="4578" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4579" max="4579" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4580" max="4580" width="10" style="13" customWidth="1"/>
+    <col min="4581" max="4581" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4582" max="4582" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4583" max="4583" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4584" max="4584" width="12.109375" style="13" customWidth="1"/>
+    <col min="4585" max="4585" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4586" max="4586" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4587" max="4587" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4588" max="4588" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4589" max="4589" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4590" max="4590" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4591" max="4591" width="9.109375" style="13" customWidth="1"/>
+    <col min="4592" max="4593" width="10" style="13" customWidth="1"/>
+    <col min="4594" max="4594" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4595" max="4832" width="8.88671875" style="13"/>
+    <col min="4833" max="4833" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4834" max="4834" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4835" max="4835" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4836" max="4836" width="10" style="13" customWidth="1"/>
+    <col min="4837" max="4837" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4838" max="4838" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4839" max="4839" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4840" max="4840" width="12.109375" style="13" customWidth="1"/>
+    <col min="4841" max="4841" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4842" max="4842" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4843" max="4843" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4844" max="4844" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4845" max="4845" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4846" max="4846" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4847" max="4847" width="9.109375" style="13" customWidth="1"/>
+    <col min="4848" max="4849" width="10" style="13" customWidth="1"/>
+    <col min="4850" max="4850" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4851" max="5088" width="8.88671875" style="13"/>
+    <col min="5089" max="5089" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5090" max="5090" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5091" max="5091" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5092" max="5092" width="10" style="13" customWidth="1"/>
+    <col min="5093" max="5093" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5094" max="5094" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5095" max="5095" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5096" max="5096" width="12.109375" style="13" customWidth="1"/>
+    <col min="5097" max="5097" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5098" max="5098" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5099" max="5099" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5100" max="5100" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5101" max="5101" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5102" max="5102" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5103" max="5103" width="9.109375" style="13" customWidth="1"/>
+    <col min="5104" max="5105" width="10" style="13" customWidth="1"/>
+    <col min="5106" max="5106" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5107" max="5344" width="8.88671875" style="13"/>
+    <col min="5345" max="5345" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5346" max="5346" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5347" max="5347" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5348" max="5348" width="10" style="13" customWidth="1"/>
+    <col min="5349" max="5349" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5350" max="5350" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5351" max="5351" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5352" max="5352" width="12.109375" style="13" customWidth="1"/>
+    <col min="5353" max="5353" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5354" max="5354" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5355" max="5355" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5356" max="5356" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5357" max="5357" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5358" max="5358" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5359" max="5359" width="9.109375" style="13" customWidth="1"/>
+    <col min="5360" max="5361" width="10" style="13" customWidth="1"/>
+    <col min="5362" max="5362" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5363" max="5600" width="8.88671875" style="13"/>
+    <col min="5601" max="5601" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5602" max="5602" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5603" max="5603" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5604" max="5604" width="10" style="13" customWidth="1"/>
+    <col min="5605" max="5605" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5606" max="5606" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5607" max="5607" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5608" max="5608" width="12.109375" style="13" customWidth="1"/>
+    <col min="5609" max="5609" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5610" max="5610" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5611" max="5611" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5612" max="5612" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5613" max="5613" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5614" max="5614" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5615" max="5615" width="9.109375" style="13" customWidth="1"/>
+    <col min="5616" max="5617" width="10" style="13" customWidth="1"/>
+    <col min="5618" max="5618" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5619" max="5856" width="8.88671875" style="13"/>
+    <col min="5857" max="5857" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5858" max="5858" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5859" max="5859" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5860" max="5860" width="10" style="13" customWidth="1"/>
+    <col min="5861" max="5861" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5862" max="5862" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5863" max="5863" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5864" max="5864" width="12.109375" style="13" customWidth="1"/>
+    <col min="5865" max="5865" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5866" max="5866" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5867" max="5867" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5868" max="5868" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5869" max="5869" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5870" max="5870" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5871" max="5871" width="9.109375" style="13" customWidth="1"/>
+    <col min="5872" max="5873" width="10" style="13" customWidth="1"/>
+    <col min="5874" max="5874" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5875" max="6112" width="8.88671875" style="13"/>
+    <col min="6113" max="6113" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6114" max="6114" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6115" max="6115" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6116" max="6116" width="10" style="13" customWidth="1"/>
+    <col min="6117" max="6117" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6118" max="6118" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6119" max="6119" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6120" max="6120" width="12.109375" style="13" customWidth="1"/>
+    <col min="6121" max="6121" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6122" max="6122" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6123" max="6123" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6124" max="6124" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6125" max="6125" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6126" max="6126" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6127" max="6127" width="9.109375" style="13" customWidth="1"/>
+    <col min="6128" max="6129" width="10" style="13" customWidth="1"/>
+    <col min="6130" max="6130" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6131" max="6368" width="8.88671875" style="13"/>
+    <col min="6369" max="6369" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6370" max="6370" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6371" max="6371" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6372" max="6372" width="10" style="13" customWidth="1"/>
+    <col min="6373" max="6373" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6374" max="6374" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6375" max="6375" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6376" max="6376" width="12.109375" style="13" customWidth="1"/>
+    <col min="6377" max="6377" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6378" max="6378" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6379" max="6379" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6380" max="6380" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6381" max="6381" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6382" max="6382" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6383" max="6383" width="9.109375" style="13" customWidth="1"/>
+    <col min="6384" max="6385" width="10" style="13" customWidth="1"/>
+    <col min="6386" max="6386" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6387" max="6624" width="8.88671875" style="13"/>
+    <col min="6625" max="6625" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6626" max="6626" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6627" max="6627" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6628" max="6628" width="10" style="13" customWidth="1"/>
+    <col min="6629" max="6629" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6630" max="6630" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6631" max="6631" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6632" max="6632" width="12.109375" style="13" customWidth="1"/>
+    <col min="6633" max="6633" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6634" max="6634" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6635" max="6635" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6636" max="6636" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6637" max="6637" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6638" max="6638" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6639" max="6639" width="9.109375" style="13" customWidth="1"/>
+    <col min="6640" max="6641" width="10" style="13" customWidth="1"/>
+    <col min="6642" max="6642" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6643" max="6880" width="8.88671875" style="13"/>
+    <col min="6881" max="6881" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6882" max="6882" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6883" max="6883" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6884" max="6884" width="10" style="13" customWidth="1"/>
+    <col min="6885" max="6885" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6886" max="6886" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6887" max="6887" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6888" max="6888" width="12.109375" style="13" customWidth="1"/>
+    <col min="6889" max="6889" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6890" max="6890" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6891" max="6891" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6892" max="6892" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6893" max="6893" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6894" max="6894" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6895" max="6895" width="9.109375" style="13" customWidth="1"/>
+    <col min="6896" max="6897" width="10" style="13" customWidth="1"/>
+    <col min="6898" max="6898" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6899" max="7136" width="8.88671875" style="13"/>
+    <col min="7137" max="7137" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7138" max="7138" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7139" max="7139" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7140" max="7140" width="10" style="13" customWidth="1"/>
+    <col min="7141" max="7141" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7142" max="7142" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7143" max="7143" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7144" max="7144" width="12.109375" style="13" customWidth="1"/>
+    <col min="7145" max="7145" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7146" max="7146" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7147" max="7147" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7148" max="7148" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7149" max="7149" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7150" max="7150" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7151" max="7151" width="9.109375" style="13" customWidth="1"/>
+    <col min="7152" max="7153" width="10" style="13" customWidth="1"/>
+    <col min="7154" max="7154" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7155" max="7392" width="8.88671875" style="13"/>
+    <col min="7393" max="7393" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7394" max="7394" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7395" max="7395" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7396" max="7396" width="10" style="13" customWidth="1"/>
+    <col min="7397" max="7397" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7398" max="7398" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7399" max="7399" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7400" max="7400" width="12.109375" style="13" customWidth="1"/>
+    <col min="7401" max="7401" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7402" max="7402" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7403" max="7403" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7404" max="7404" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7405" max="7405" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7406" max="7406" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7407" max="7407" width="9.109375" style="13" customWidth="1"/>
+    <col min="7408" max="7409" width="10" style="13" customWidth="1"/>
+    <col min="7410" max="7410" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7411" max="7648" width="8.88671875" style="13"/>
+    <col min="7649" max="7649" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7650" max="7650" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7651" max="7651" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7652" max="7652" width="10" style="13" customWidth="1"/>
+    <col min="7653" max="7653" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7654" max="7654" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7655" max="7655" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7656" max="7656" width="12.109375" style="13" customWidth="1"/>
+    <col min="7657" max="7657" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7658" max="7658" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7659" max="7659" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7660" max="7660" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7661" max="7661" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7662" max="7662" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7663" max="7663" width="9.109375" style="13" customWidth="1"/>
+    <col min="7664" max="7665" width="10" style="13" customWidth="1"/>
+    <col min="7666" max="7666" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7667" max="7904" width="8.88671875" style="13"/>
+    <col min="7905" max="7905" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7906" max="7906" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7907" max="7907" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7908" max="7908" width="10" style="13" customWidth="1"/>
+    <col min="7909" max="7909" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7910" max="7910" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7911" max="7911" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7912" max="7912" width="12.109375" style="13" customWidth="1"/>
+    <col min="7913" max="7913" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7914" max="7914" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7915" max="7915" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7916" max="7916" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7917" max="7917" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7918" max="7918" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7919" max="7919" width="9.109375" style="13" customWidth="1"/>
+    <col min="7920" max="7921" width="10" style="13" customWidth="1"/>
+    <col min="7922" max="7922" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7923" max="8160" width="8.88671875" style="13"/>
+    <col min="8161" max="8161" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8162" max="8162" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8163" max="8163" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8164" max="8164" width="10" style="13" customWidth="1"/>
+    <col min="8165" max="8165" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8166" max="8166" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8167" max="8167" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8168" max="8168" width="12.109375" style="13" customWidth="1"/>
+    <col min="8169" max="8169" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8170" max="8170" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8171" max="8171" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8172" max="8172" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8173" max="8173" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8174" max="8174" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8175" max="8175" width="9.109375" style="13" customWidth="1"/>
+    <col min="8176" max="8177" width="10" style="13" customWidth="1"/>
+    <col min="8178" max="8178" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8179" max="8416" width="8.88671875" style="13"/>
+    <col min="8417" max="8417" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8418" max="8418" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8419" max="8419" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8420" max="8420" width="10" style="13" customWidth="1"/>
+    <col min="8421" max="8421" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8422" max="8422" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8423" max="8423" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8424" max="8424" width="12.109375" style="13" customWidth="1"/>
+    <col min="8425" max="8425" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8426" max="8426" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8427" max="8427" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8428" max="8428" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8429" max="8429" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8430" max="8430" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8431" max="8431" width="9.109375" style="13" customWidth="1"/>
+    <col min="8432" max="8433" width="10" style="13" customWidth="1"/>
+    <col min="8434" max="8434" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8435" max="8672" width="8.88671875" style="13"/>
+    <col min="8673" max="8673" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8674" max="8674" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8675" max="8675" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8676" max="8676" width="10" style="13" customWidth="1"/>
+    <col min="8677" max="8677" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8678" max="8678" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8679" max="8679" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8680" max="8680" width="12.109375" style="13" customWidth="1"/>
+    <col min="8681" max="8681" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8682" max="8682" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8683" max="8683" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8684" max="8684" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8685" max="8685" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8686" max="8686" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8687" max="8687" width="9.109375" style="13" customWidth="1"/>
+    <col min="8688" max="8689" width="10" style="13" customWidth="1"/>
+    <col min="8690" max="8690" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8691" max="8928" width="8.88671875" style="13"/>
+    <col min="8929" max="8929" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8930" max="8930" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8931" max="8931" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8932" max="8932" width="10" style="13" customWidth="1"/>
+    <col min="8933" max="8933" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8934" max="8934" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8935" max="8935" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8936" max="8936" width="12.109375" style="13" customWidth="1"/>
+    <col min="8937" max="8937" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8938" max="8938" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8939" max="8939" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8940" max="8940" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8941" max="8941" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8942" max="8942" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8943" max="8943" width="9.109375" style="13" customWidth="1"/>
+    <col min="8944" max="8945" width="10" style="13" customWidth="1"/>
+    <col min="8946" max="8946" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8947" max="9184" width="8.88671875" style="13"/>
+    <col min="9185" max="9185" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9186" max="9186" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9187" max="9187" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9188" max="9188" width="10" style="13" customWidth="1"/>
+    <col min="9189" max="9189" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9190" max="9190" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9191" max="9191" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9192" max="9192" width="12.109375" style="13" customWidth="1"/>
+    <col min="9193" max="9193" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9194" max="9194" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9195" max="9195" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9196" max="9196" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9197" max="9197" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9198" max="9198" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9199" max="9199" width="9.109375" style="13" customWidth="1"/>
+    <col min="9200" max="9201" width="10" style="13" customWidth="1"/>
+    <col min="9202" max="9202" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9203" max="9440" width="8.88671875" style="13"/>
+    <col min="9441" max="9441" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9442" max="9442" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9443" max="9443" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9444" max="9444" width="10" style="13" customWidth="1"/>
+    <col min="9445" max="9445" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9446" max="9446" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9447" max="9447" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9448" max="9448" width="12.109375" style="13" customWidth="1"/>
+    <col min="9449" max="9449" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9450" max="9450" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9451" max="9451" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9452" max="9452" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9453" max="9453" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9454" max="9454" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9455" max="9455" width="9.109375" style="13" customWidth="1"/>
+    <col min="9456" max="9457" width="10" style="13" customWidth="1"/>
+    <col min="9458" max="9458" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9459" max="9696" width="8.88671875" style="13"/>
+    <col min="9697" max="9697" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9698" max="9698" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9699" max="9699" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9700" max="9700" width="10" style="13" customWidth="1"/>
+    <col min="9701" max="9701" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9702" max="9702" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9703" max="9703" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9704" max="9704" width="12.109375" style="13" customWidth="1"/>
+    <col min="9705" max="9705" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9706" max="9706" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9707" max="9707" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9708" max="9708" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9709" max="9709" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9710" max="9710" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9711" max="9711" width="9.109375" style="13" customWidth="1"/>
+    <col min="9712" max="9713" width="10" style="13" customWidth="1"/>
+    <col min="9714" max="9714" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9715" max="9952" width="8.88671875" style="13"/>
+    <col min="9953" max="9953" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9954" max="9954" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9955" max="9955" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9956" max="9956" width="10" style="13" customWidth="1"/>
+    <col min="9957" max="9957" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9958" max="9958" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9959" max="9959" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9960" max="9960" width="12.109375" style="13" customWidth="1"/>
+    <col min="9961" max="9961" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9962" max="9962" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9963" max="9963" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9964" max="9964" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9965" max="9965" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9966" max="9966" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9967" max="9967" width="9.109375" style="13" customWidth="1"/>
+    <col min="9968" max="9969" width="10" style="13" customWidth="1"/>
+    <col min="9970" max="9970" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9971" max="10208" width="8.88671875" style="13"/>
+    <col min="10209" max="10209" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10210" max="10210" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10211" max="10211" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10212" max="10212" width="10" style="13" customWidth="1"/>
+    <col min="10213" max="10213" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10214" max="10214" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10215" max="10215" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10216" max="10216" width="12.109375" style="13" customWidth="1"/>
+    <col min="10217" max="10217" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10218" max="10218" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10219" max="10219" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10220" max="10220" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10221" max="10221" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10222" max="10222" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10223" max="10223" width="9.109375" style="13" customWidth="1"/>
+    <col min="10224" max="10225" width="10" style="13" customWidth="1"/>
+    <col min="10226" max="10226" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10227" max="10464" width="8.88671875" style="13"/>
+    <col min="10465" max="10465" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10466" max="10466" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10467" max="10467" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10468" max="10468" width="10" style="13" customWidth="1"/>
+    <col min="10469" max="10469" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10470" max="10470" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10471" max="10471" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10472" max="10472" width="12.109375" style="13" customWidth="1"/>
+    <col min="10473" max="10473" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10474" max="10474" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10475" max="10475" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10476" max="10476" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10477" max="10477" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10478" max="10478" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10479" max="10479" width="9.109375" style="13" customWidth="1"/>
+    <col min="10480" max="10481" width="10" style="13" customWidth="1"/>
+    <col min="10482" max="10482" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10483" max="10720" width="8.88671875" style="13"/>
+    <col min="10721" max="10721" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10722" max="10722" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10723" max="10723" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10724" max="10724" width="10" style="13" customWidth="1"/>
+    <col min="10725" max="10725" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10726" max="10726" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10727" max="10727" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10728" max="10728" width="12.109375" style="13" customWidth="1"/>
+    <col min="10729" max="10729" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10730" max="10730" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10731" max="10731" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10732" max="10732" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10733" max="10733" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10734" max="10734" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10735" max="10735" width="9.109375" style="13" customWidth="1"/>
+    <col min="10736" max="10737" width="10" style="13" customWidth="1"/>
+    <col min="10738" max="10738" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10739" max="10976" width="8.88671875" style="13"/>
+    <col min="10977" max="10977" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10978" max="10978" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10979" max="10979" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10980" max="10980" width="10" style="13" customWidth="1"/>
+    <col min="10981" max="10981" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10982" max="10982" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10983" max="10983" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10984" max="10984" width="12.109375" style="13" customWidth="1"/>
+    <col min="10985" max="10985" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10986" max="10986" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10987" max="10987" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10988" max="10988" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10989" max="10989" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10990" max="10990" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10991" max="10991" width="9.109375" style="13" customWidth="1"/>
+    <col min="10992" max="10993" width="10" style="13" customWidth="1"/>
+    <col min="10994" max="10994" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10995" max="11232" width="8.88671875" style="13"/>
+    <col min="11233" max="11233" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11234" max="11234" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11235" max="11235" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11236" max="11236" width="10" style="13" customWidth="1"/>
+    <col min="11237" max="11237" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11238" max="11238" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11239" max="11239" width="13.44140625" style="13" customWidth="1"/>
+    <col min="11240" max="11240" width="12.109375" style="13" customWidth="1"/>
+    <col min="11241" max="11241" width="11.88671875" style="13" customWidth="1"/>
+    <col min="11242" max="11242" width="12.44140625" style="13" customWidth="1"/>
+    <col min="11243" max="11243" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11244" max="11244" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11245" max="11245" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11246" max="11246" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11247" max="11247" width="9.109375" style="13" customWidth="1"/>
+    <col min="11248" max="11249" width="10" style="13" customWidth="1"/>
+    <col min="11250" max="11250" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11251" max="11488" width="8.88671875" style="13"/>
+    <col min="11489" max="11489" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11490" max="11490" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11491" max="11491" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11492" max="11492" width="10" style="13" customWidth="1"/>
+    <col min="11493" max="11493" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11494" max="11494" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11495" max="11495" width="13.44140625" style="13" customWidth="1"/>
+    <col min="11496" max="11496" width="12.109375" style="13" customWidth="1"/>
+    <col min="11497" max="11497" width="11.88671875" style="13" customWidth="1"/>
+    <col min="11498" max="11498" width="12.44140625" style="13" customWidth="1"/>
+    <col min="11499" max="11499" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11500" max="11500" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11501" max="11501" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11502" max="11502" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11503" max="11503" width="9.109375" style="13" customWidth="1"/>
+    <col min="11504" max="11505" width="10" style="13" customWidth="1"/>
+    <col min="11506" max="11506" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11507" max="11744" width="8.88671875" style="13"/>
+    <col min="11745" max="11745" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11746" max="11746" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11747" max="11747" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11748" max="11748" width="10" style="13" customWidth="1"/>
+    <col min="11749" max="11749" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11750" max="11750" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11751" max="11751" width="13.44140625" style="13" customWidth="1"/>
+    <col min="11752" max="11752" width="12.109375" style="13" customWidth="1"/>
+    <col min="11753" max="11753" width="11.88671875" style="13" customWidth="1"/>
+    <col min="11754" max="11754" width="12.44140625" style="13" customWidth="1"/>
+    <col min="11755" max="11755" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11756" max="11756" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11757" max="11757" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11758" max="11758" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11759" max="11759" width="9.109375" style="13" customWidth="1"/>
+    <col min="11760" max="11761" width="10" style="13" customWidth="1"/>
+    <col min="11762" max="11762" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11763" max="12000" width="8.88671875" style="13"/>
+    <col min="12001" max="12001" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12002" max="12002" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12003" max="12003" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12004" max="12004" width="10" style="13" customWidth="1"/>
+    <col min="12005" max="12005" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12006" max="12006" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12007" max="12007" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12008" max="12008" width="12.109375" style="13" customWidth="1"/>
+    <col min="12009" max="12009" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12010" max="12010" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12011" max="12011" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12012" max="12012" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12013" max="12013" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12014" max="12014" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12015" max="12015" width="9.109375" style="13" customWidth="1"/>
+    <col min="12016" max="12017" width="10" style="13" customWidth="1"/>
+    <col min="12018" max="12018" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12019" max="12256" width="8.88671875" style="13"/>
+    <col min="12257" max="12257" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12258" max="12258" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12259" max="12259" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12260" max="12260" width="10" style="13" customWidth="1"/>
+    <col min="12261" max="12261" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12262" max="12262" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12263" max="12263" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12264" max="12264" width="12.109375" style="13" customWidth="1"/>
+    <col min="12265" max="12265" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12266" max="12266" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12267" max="12267" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12268" max="12268" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12269" max="12269" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12270" max="12270" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12271" max="12271" width="9.109375" style="13" customWidth="1"/>
+    <col min="12272" max="12273" width="10" style="13" customWidth="1"/>
+    <col min="12274" max="12274" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12275" max="12512" width="8.88671875" style="13"/>
+    <col min="12513" max="12513" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12514" max="12514" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12515" max="12515" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12516" max="12516" width="10" style="13" customWidth="1"/>
+    <col min="12517" max="12517" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12518" max="12518" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12519" max="12519" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12520" max="12520" width="12.109375" style="13" customWidth="1"/>
+    <col min="12521" max="12521" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12522" max="12522" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12523" max="12523" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12524" max="12524" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12525" max="12525" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12526" max="12526" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12527" max="12527" width="9.109375" style="13" customWidth="1"/>
+    <col min="12528" max="12529" width="10" style="13" customWidth="1"/>
+    <col min="12530" max="12530" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12531" max="12768" width="8.88671875" style="13"/>
+    <col min="12769" max="12769" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12770" max="12770" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12771" max="12771" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12772" max="12772" width="10" style="13" customWidth="1"/>
+    <col min="12773" max="12773" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12774" max="12774" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12775" max="12775" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12776" max="12776" width="12.109375" style="13" customWidth="1"/>
+    <col min="12777" max="12777" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12778" max="12778" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12779" max="12779" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12780" max="12780" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12781" max="12781" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12782" max="12782" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12783" max="12783" width="9.109375" style="13" customWidth="1"/>
+    <col min="12784" max="12785" width="10" style="13" customWidth="1"/>
+    <col min="12786" max="12786" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12787" max="13024" width="8.88671875" style="13"/>
+    <col min="13025" max="13025" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13026" max="13026" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13027" max="13027" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13028" max="13028" width="10" style="13" customWidth="1"/>
+    <col min="13029" max="13029" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13030" max="13030" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13031" max="13031" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13032" max="13032" width="12.109375" style="13" customWidth="1"/>
+    <col min="13033" max="13033" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13034" max="13034" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13035" max="13035" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13036" max="13036" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13037" max="13037" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13038" max="13038" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13039" max="13039" width="9.109375" style="13" customWidth="1"/>
+    <col min="13040" max="13041" width="10" style="13" customWidth="1"/>
+    <col min="13042" max="13042" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13043" max="13280" width="8.88671875" style="13"/>
+    <col min="13281" max="13281" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13282" max="13282" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13283" max="13283" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13284" max="13284" width="10" style="13" customWidth="1"/>
+    <col min="13285" max="13285" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13286" max="13286" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13287" max="13287" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13288" max="13288" width="12.109375" style="13" customWidth="1"/>
+    <col min="13289" max="13289" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13290" max="13290" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13291" max="13291" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13292" max="13292" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13293" max="13293" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13294" max="13294" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13295" max="13295" width="9.109375" style="13" customWidth="1"/>
+    <col min="13296" max="13297" width="10" style="13" customWidth="1"/>
+    <col min="13298" max="13298" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13299" max="13536" width="8.88671875" style="13"/>
+    <col min="13537" max="13537" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13538" max="13538" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13539" max="13539" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13540" max="13540" width="10" style="13" customWidth="1"/>
+    <col min="13541" max="13541" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13542" max="13542" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13543" max="13543" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13544" max="13544" width="12.109375" style="13" customWidth="1"/>
+    <col min="13545" max="13545" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13546" max="13546" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13547" max="13547" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13548" max="13548" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13549" max="13549" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13550" max="13550" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13551" max="13551" width="9.109375" style="13" customWidth="1"/>
+    <col min="13552" max="13553" width="10" style="13" customWidth="1"/>
+    <col min="13554" max="13554" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13555" max="13792" width="8.88671875" style="13"/>
+    <col min="13793" max="13793" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13794" max="13794" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13795" max="13795" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13796" max="13796" width="10" style="13" customWidth="1"/>
+    <col min="13797" max="13797" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13798" max="13798" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13799" max="13799" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13800" max="13800" width="12.109375" style="13" customWidth="1"/>
+    <col min="13801" max="13801" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13802" max="13802" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13803" max="13803" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13804" max="13804" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13805" max="13805" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13806" max="13806" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13807" max="13807" width="9.109375" style="13" customWidth="1"/>
+    <col min="13808" max="13809" width="10" style="13" customWidth="1"/>
+    <col min="13810" max="13810" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13811" max="14048" width="8.88671875" style="13"/>
+    <col min="14049" max="14049" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14050" max="14050" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14051" max="14051" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14052" max="14052" width="10" style="13" customWidth="1"/>
+    <col min="14053" max="14053" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14054" max="14054" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14055" max="14055" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14056" max="14056" width="12.109375" style="13" customWidth="1"/>
+    <col min="14057" max="14057" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14058" max="14058" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14059" max="14059" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14060" max="14060" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14061" max="14061" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14062" max="14062" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14063" max="14063" width="9.109375" style="13" customWidth="1"/>
+    <col min="14064" max="14065" width="10" style="13" customWidth="1"/>
+    <col min="14066" max="14066" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14067" max="14304" width="8.88671875" style="13"/>
+    <col min="14305" max="14305" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14306" max="14306" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14307" max="14307" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14308" max="14308" width="10" style="13" customWidth="1"/>
+    <col min="14309" max="14309" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14310" max="14310" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14311" max="14311" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14312" max="14312" width="12.109375" style="13" customWidth="1"/>
+    <col min="14313" max="14313" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14314" max="14314" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14315" max="14315" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14316" max="14316" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14317" max="14317" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14318" max="14318" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14319" max="14319" width="9.109375" style="13" customWidth="1"/>
+    <col min="14320" max="14321" width="10" style="13" customWidth="1"/>
+    <col min="14322" max="14322" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14323" max="14560" width="8.88671875" style="13"/>
+    <col min="14561" max="14561" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14562" max="14562" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14563" max="14563" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14564" max="14564" width="10" style="13" customWidth="1"/>
+    <col min="14565" max="14565" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14566" max="14566" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14567" max="14567" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14568" max="14568" width="12.109375" style="13" customWidth="1"/>
+    <col min="14569" max="14569" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14570" max="14570" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14571" max="14571" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14572" max="14572" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14573" max="14573" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14574" max="14574" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14575" max="14575" width="9.109375" style="13" customWidth="1"/>
+    <col min="14576" max="14577" width="10" style="13" customWidth="1"/>
+    <col min="14578" max="14578" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14579" max="14816" width="8.88671875" style="13"/>
+    <col min="14817" max="14817" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14818" max="14818" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14819" max="14819" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14820" max="14820" width="10" style="13" customWidth="1"/>
+    <col min="14821" max="14821" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14822" max="14822" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14823" max="14823" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14824" max="14824" width="12.109375" style="13" customWidth="1"/>
+    <col min="14825" max="14825" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14826" max="14826" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14827" max="14827" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14828" max="14828" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14829" max="14829" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14830" max="14830" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14831" max="14831" width="9.109375" style="13" customWidth="1"/>
+    <col min="14832" max="14833" width="10" style="13" customWidth="1"/>
+    <col min="14834" max="14834" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14835" max="15072" width="8.88671875" style="13"/>
+    <col min="15073" max="15073" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15074" max="15074" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15075" max="15075" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15076" max="15076" width="10" style="13" customWidth="1"/>
+    <col min="15077" max="15077" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15078" max="15078" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15079" max="15079" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15080" max="15080" width="12.109375" style="13" customWidth="1"/>
+    <col min="15081" max="15081" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15082" max="15082" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15083" max="15083" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15084" max="15084" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15085" max="15085" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15086" max="15086" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15087" max="15087" width="9.109375" style="13" customWidth="1"/>
+    <col min="15088" max="15089" width="10" style="13" customWidth="1"/>
+    <col min="15090" max="15090" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15091" max="15328" width="8.88671875" style="13"/>
+    <col min="15329" max="15329" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15330" max="15330" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15331" max="15331" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15332" max="15332" width="10" style="13" customWidth="1"/>
+    <col min="15333" max="15333" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15334" max="15334" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15335" max="15335" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15336" max="15336" width="12.109375" style="13" customWidth="1"/>
+    <col min="15337" max="15337" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15338" max="15338" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15339" max="15339" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15340" max="15340" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15341" max="15341" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15342" max="15342" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15343" max="15343" width="9.109375" style="13" customWidth="1"/>
+    <col min="15344" max="15345" width="10" style="13" customWidth="1"/>
+    <col min="15346" max="15346" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15347" max="15584" width="8.88671875" style="13"/>
+    <col min="15585" max="15585" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15586" max="15586" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15587" max="15587" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15588" max="15588" width="10" style="13" customWidth="1"/>
+    <col min="15589" max="15589" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15590" max="15590" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15591" max="15591" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15592" max="15592" width="12.109375" style="13" customWidth="1"/>
+    <col min="15593" max="15593" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15594" max="15594" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15595" max="15595" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15596" max="15596" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15597" max="15597" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15598" max="15598" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15599" max="15599" width="9.109375" style="13" customWidth="1"/>
+    <col min="15600" max="15601" width="10" style="13" customWidth="1"/>
+    <col min="15602" max="15602" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15603" max="15840" width="8.88671875" style="13"/>
+    <col min="15841" max="15841" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15842" max="15842" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15843" max="15843" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15844" max="15844" width="10" style="13" customWidth="1"/>
+    <col min="15845" max="15845" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15846" max="15846" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15847" max="15847" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15848" max="15848" width="12.109375" style="13" customWidth="1"/>
+    <col min="15849" max="15849" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15850" max="15850" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15851" max="15851" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15852" max="15852" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15853" max="15853" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15854" max="15854" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15855" max="15855" width="9.109375" style="13" customWidth="1"/>
+    <col min="15856" max="15857" width="10" style="13" customWidth="1"/>
+    <col min="15858" max="15858" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15859" max="16096" width="8.88671875" style="13"/>
+    <col min="16097" max="16097" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16098" max="16098" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16099" max="16099" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16100" max="16100" width="10" style="13" customWidth="1"/>
+    <col min="16101" max="16101" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="16102" max="16102" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16103" max="16103" width="13.44140625" style="13" customWidth="1"/>
+    <col min="16104" max="16104" width="12.109375" style="13" customWidth="1"/>
+    <col min="16105" max="16105" width="11.88671875" style="13" customWidth="1"/>
+    <col min="16106" max="16106" width="12.44140625" style="13" customWidth="1"/>
+    <col min="16107" max="16107" width="11.44140625" style="13" customWidth="1"/>
+    <col min="16108" max="16108" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="16109" max="16109" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16110" max="16110" width="11.44140625" style="13" customWidth="1"/>
+    <col min="16111" max="16111" width="9.109375" style="13" customWidth="1"/>
+    <col min="16112" max="16113" width="10" style="13" customWidth="1"/>
+    <col min="16114" max="16114" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16115" max="16384" width="8.88671875" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="53">
+        <v>44835</v>
+      </c>
+      <c r="D1" s="53">
+        <v>44927</v>
+      </c>
+      <c r="E1" s="53">
+        <v>45017</v>
+      </c>
+      <c r="F1" s="53">
+        <v>45108</v>
+      </c>
+      <c r="G1" s="53">
+        <v>45200</v>
+      </c>
+      <c r="H1" s="53">
+        <v>45292</v>
+      </c>
+      <c r="I1" s="53">
+        <v>45383</v>
+      </c>
+      <c r="J1" s="53">
+        <v>45474</v>
+      </c>
+      <c r="K1" s="53">
+        <v>45566</v>
+      </c>
+      <c r="L1" s="53">
+        <v>45658</v>
+      </c>
+      <c r="M1" s="53">
+        <v>45748</v>
+      </c>
+      <c r="N1" s="53">
+        <v>45839</v>
+      </c>
+      <c r="O1" s="53">
+        <v>45931</v>
+      </c>
+      <c r="P1" s="53">
+        <v>46023</v>
+      </c>
+      <c r="Q1" s="53">
+        <v>46113</v>
+      </c>
+      <c r="R1" s="53">
+        <v>46204</v>
+      </c>
+      <c r="S1" s="53">
+        <v>46296</v>
+      </c>
+      <c r="T1" s="53">
+        <v>46388</v>
+      </c>
+      <c r="U1" s="53">
+        <v>46478</v>
+      </c>
+      <c r="V1" s="53">
+        <v>46569</v>
+      </c>
+      <c r="W1" s="53">
+        <v>46661</v>
+      </c>
+      <c r="X1" s="53">
+        <v>46753</v>
+      </c>
+      <c r="Y1" s="53">
+        <v>46844</v>
+      </c>
+      <c r="Z1" s="53">
+        <v>46935</v>
+      </c>
+      <c r="AA1" s="53">
+        <v>47027</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="41">
+        <v>1250</v>
+      </c>
+      <c r="D2" s="41">
+        <v>1250</v>
+      </c>
+      <c r="E2" s="41">
+        <v>1250</v>
+      </c>
+      <c r="F2" s="41">
+        <v>1250</v>
+      </c>
+      <c r="G2" s="41">
+        <v>1250</v>
+      </c>
+      <c r="H2" s="41">
+        <v>1400</v>
+      </c>
+      <c r="I2" s="41">
+        <v>1400</v>
+      </c>
+      <c r="J2" s="41">
+        <v>1400</v>
+      </c>
+      <c r="K2" s="41">
+        <v>1400</v>
+      </c>
+      <c r="L2" s="41">
+        <v>1700</v>
+      </c>
+      <c r="M2" s="41">
+        <v>1700</v>
+      </c>
+      <c r="N2" s="41">
+        <v>1700</v>
+      </c>
+      <c r="O2" s="41">
+        <v>1700</v>
+      </c>
+      <c r="P2" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="41">
+        <f t="shared" ref="Q2:AA2" ca="1" si="0">P2*(RAND()*(1.04-1.025)+1.025)</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Y2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA2" s="41">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="41">
+        <v>240</v>
+      </c>
+      <c r="D3" s="41">
+        <v>240</v>
+      </c>
+      <c r="E3" s="41">
+        <v>240</v>
+      </c>
+      <c r="F3" s="41">
+        <v>240</v>
+      </c>
+      <c r="G3" s="41">
+        <v>240</v>
+      </c>
+      <c r="H3" s="41">
+        <v>270</v>
+      </c>
+      <c r="I3" s="41">
+        <v>270</v>
+      </c>
+      <c r="J3" s="41">
+        <v>270</v>
+      </c>
+      <c r="K3" s="41">
+        <v>270</v>
+      </c>
+      <c r="L3" s="41">
+        <v>270</v>
+      </c>
+      <c r="M3" s="41">
+        <v>270</v>
+      </c>
+      <c r="N3" s="41">
+        <v>270</v>
+      </c>
+      <c r="O3" s="41">
+        <v>270</v>
+      </c>
+      <c r="P3" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="41">
+        <f t="shared" ref="Q3:AA4" ca="1" si="1">P3*(RAND()*(1.15-0.93)+0.93)</f>
+        <v>0</v>
+      </c>
+      <c r="R3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="W3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="X3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AA3" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="41">
+        <v>3100</v>
+      </c>
+      <c r="D4" s="41">
+        <v>3100</v>
+      </c>
+      <c r="E4" s="41">
+        <v>3100</v>
+      </c>
+      <c r="F4" s="41">
+        <v>3100</v>
+      </c>
+      <c r="G4" s="41">
+        <v>3100</v>
+      </c>
+      <c r="H4" s="41">
+        <v>4500</v>
+      </c>
+      <c r="I4" s="41">
+        <v>4500</v>
+      </c>
+      <c r="J4" s="41">
+        <v>4500</v>
+      </c>
+      <c r="K4" s="41">
+        <v>4500</v>
+      </c>
+      <c r="L4" s="41">
+        <v>5300</v>
+      </c>
+      <c r="M4" s="41">
+        <v>5900</v>
+      </c>
+      <c r="N4" s="41">
+        <v>6200</v>
+      </c>
+      <c r="O4" s="41">
+        <v>6900</v>
+      </c>
+      <c r="P4" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="R4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="W4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="X4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AA4" s="41">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="41">
+        <v>140</v>
+      </c>
+      <c r="D5" s="41">
+        <v>140</v>
+      </c>
+      <c r="E5" s="41">
+        <v>140</v>
+      </c>
+      <c r="F5" s="41">
+        <v>140</v>
+      </c>
+      <c r="G5" s="41">
+        <v>140</v>
+      </c>
+      <c r="H5" s="41">
+        <v>140</v>
+      </c>
+      <c r="I5" s="41">
+        <v>140</v>
+      </c>
+      <c r="J5" s="41">
+        <v>140</v>
+      </c>
+      <c r="K5" s="41">
+        <v>140</v>
+      </c>
+      <c r="L5" s="41">
+        <v>160</v>
+      </c>
+      <c r="M5" s="41">
+        <v>160.55219753626932</v>
+      </c>
+      <c r="N5" s="41">
+        <v>160.55219753626932</v>
+      </c>
+      <c r="O5" s="41">
+        <v>160.55219753626932</v>
+      </c>
+      <c r="P5" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="41">
+        <f t="shared" ref="Q5:AA5" ca="1" si="2">P5*(RAND()*(1.05-1.1)+1.05)</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="41">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="41">
+        <v>450</v>
+      </c>
+      <c r="D6" s="41">
+        <v>450</v>
+      </c>
+      <c r="E6" s="41">
+        <v>450</v>
+      </c>
+      <c r="F6" s="41">
+        <v>450</v>
+      </c>
+      <c r="G6" s="41">
+        <v>450</v>
+      </c>
+      <c r="H6" s="41">
+        <v>550</v>
+      </c>
+      <c r="I6" s="41">
+        <v>550</v>
+      </c>
+      <c r="J6" s="41">
+        <v>550</v>
+      </c>
+      <c r="K6" s="41">
+        <v>550</v>
+      </c>
+      <c r="L6" s="41">
+        <v>600</v>
+      </c>
+      <c r="M6" s="41">
+        <v>600</v>
+      </c>
+      <c r="N6" s="41">
+        <v>600</v>
+      </c>
+      <c r="O6" s="41">
+        <v>600</v>
+      </c>
+      <c r="P6" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="41">
+        <f t="shared" ref="Q6:AA6" ca="1" si="3">P6*(RAND()*(1.05-1.01)+1.01)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="T6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="V6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="W6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="41">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="D7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="E7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="F7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="G7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="H7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="I7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="J7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="K7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="L7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="M7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="N7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="O7" s="41">
+        <v>64.12</v>
+      </c>
+      <c r="P7" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="41">
+        <v>0</v>
+      </c>
+      <c r="R7" s="41">
+        <v>0</v>
+      </c>
+      <c r="S7" s="41">
+        <v>0</v>
+      </c>
+      <c r="T7" s="41">
+        <v>0</v>
+      </c>
+      <c r="U7" s="41">
+        <v>0</v>
+      </c>
+      <c r="V7" s="41">
+        <v>0</v>
+      </c>
+      <c r="W7" s="41">
+        <v>0</v>
+      </c>
+      <c r="X7" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="41">
+        <v>650</v>
+      </c>
+      <c r="D8" s="41">
+        <v>650</v>
+      </c>
+      <c r="E8" s="41">
+        <v>650</v>
+      </c>
+      <c r="F8" s="41">
+        <v>650</v>
+      </c>
+      <c r="G8" s="41">
+        <v>650</v>
+      </c>
+      <c r="H8" s="41">
+        <v>750</v>
+      </c>
+      <c r="I8" s="41">
+        <v>750</v>
+      </c>
+      <c r="J8" s="41">
+        <v>750</v>
+      </c>
+      <c r="K8" s="41">
+        <v>750</v>
+      </c>
+      <c r="L8" s="41">
+        <v>830</v>
+      </c>
+      <c r="M8" s="41">
+        <v>830</v>
+      </c>
+      <c r="N8" s="41">
+        <v>830</v>
+      </c>
+      <c r="O8" s="41">
+        <v>830</v>
+      </c>
+      <c r="P8" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="41">
+        <f t="shared" ref="Q8:AA8" ca="1" si="4">P8*(RAND()*(1.04-1.025)+1.025)</f>
+        <v>0</v>
+      </c>
+      <c r="R8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="S8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="U8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="W8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="X8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AA8" s="41">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="41">
+        <f>'Cash Flow Statement_Budget'!B3*0.003</f>
+        <v>385.80014922061724</v>
+      </c>
+      <c r="D9" s="41">
+        <v>733.68749605800008</v>
+      </c>
+      <c r="E9" s="41">
+        <v>965.50834941599987</v>
+      </c>
+      <c r="F9" s="41">
+        <v>755.10175226399997</v>
+      </c>
+      <c r="G9" s="41">
+        <v>648.81721488000017</v>
+      </c>
+      <c r="H9" s="41">
+        <v>866.55734519999999</v>
+      </c>
+      <c r="I9" s="41">
+        <v>957.69059879999998</v>
+      </c>
+      <c r="J9" s="41">
+        <v>828.30601379999996</v>
+      </c>
+      <c r="K9" s="41">
+        <v>608.79067508555295</v>
+      </c>
+      <c r="L9" s="41">
+        <v>977.54154885360003</v>
+      </c>
+      <c r="M9" s="41">
+        <v>1315.0039020013139</v>
+      </c>
+      <c r="N9" s="41">
+        <v>856.92771477797896</v>
+      </c>
+      <c r="O9" s="41">
+        <v>772.57751519999999</v>
+      </c>
+      <c r="P9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!O3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="Q9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!P3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="R9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!Q3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="S9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!R3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="T9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!S3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="U9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!T3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="V9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!U3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="W9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!V3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="X9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!W3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="Y9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!X3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!Y3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="AA9" s="41">
+        <f>'[1]Cash Flow Statement_Actual'!Z3*0.003</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="D10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="E10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="F10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="G10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="H10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="I10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="J10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="K10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="L10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="M10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="N10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="O10" s="41">
+        <v>248.6</v>
+      </c>
+      <c r="P10" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="41">
+        <f t="shared" ref="Q10:AA10" ca="1" si="5">P10*(RAND()*(1.04-1.025)+1.025)</f>
+        <v>0</v>
+      </c>
+      <c r="R10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="S10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="V10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="X10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Y10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Z10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AA10" s="41">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="41">
+        <v>90</v>
+      </c>
+      <c r="D11" s="41">
+        <v>90</v>
+      </c>
+      <c r="E11" s="41">
+        <v>90</v>
+      </c>
+      <c r="F11" s="41">
+        <v>90</v>
+      </c>
+      <c r="G11" s="41">
+        <v>90</v>
+      </c>
+      <c r="H11" s="41">
+        <v>120</v>
+      </c>
+      <c r="I11" s="41">
+        <v>120</v>
+      </c>
+      <c r="J11" s="41">
+        <v>120</v>
+      </c>
+      <c r="K11" s="41">
+        <v>120</v>
+      </c>
+      <c r="L11" s="41">
+        <v>140</v>
+      </c>
+      <c r="M11" s="41">
+        <v>140</v>
+      </c>
+      <c r="N11" s="41">
+        <v>140</v>
+      </c>
+      <c r="O11" s="41">
+        <v>140</v>
+      </c>
+      <c r="P11" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="41">
+        <v>0</v>
+      </c>
+      <c r="R11" s="41">
+        <v>0</v>
+      </c>
+      <c r="S11" s="41">
+        <v>0</v>
+      </c>
+      <c r="T11" s="41">
+        <v>0</v>
+      </c>
+      <c r="U11" s="41">
+        <v>0</v>
+      </c>
+      <c r="V11" s="41">
+        <v>0</v>
+      </c>
+      <c r="W11" s="41">
+        <v>0</v>
+      </c>
+      <c r="X11" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="41">
+        <v>10000</v>
+      </c>
+      <c r="D12" s="41">
+        <v>20000</v>
+      </c>
+      <c r="E12" s="41">
+        <v>20000</v>
+      </c>
+      <c r="F12" s="41">
+        <v>17000</v>
+      </c>
+      <c r="G12" s="41">
+        <v>15000</v>
+      </c>
+      <c r="H12" s="41">
+        <v>24000</v>
+      </c>
+      <c r="I12" s="41">
+        <v>23000</v>
+      </c>
+      <c r="J12" s="41">
+        <v>18000</v>
+      </c>
+      <c r="K12" s="41">
+        <v>9000</v>
+      </c>
+      <c r="L12" s="41">
+        <v>27000</v>
+      </c>
+      <c r="M12" s="41">
+        <v>25000</v>
+      </c>
+      <c r="N12" s="41">
+        <v>19000</v>
+      </c>
+      <c r="O12" s="41">
+        <v>16000</v>
+      </c>
+      <c r="P12" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="41">
+        <v>0</v>
+      </c>
+      <c r="R12" s="41">
+        <v>0</v>
+      </c>
+      <c r="S12" s="41">
+        <v>0</v>
+      </c>
+      <c r="T12" s="41">
+        <v>0</v>
+      </c>
+      <c r="U12" s="41">
+        <v>0</v>
+      </c>
+      <c r="V12" s="41">
+        <v>0</v>
+      </c>
+      <c r="W12" s="41">
+        <v>0</v>
+      </c>
+      <c r="X12" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="41">
+        <v>200</v>
+      </c>
+      <c r="D13" s="41">
+        <v>200</v>
+      </c>
+      <c r="E13" s="41">
+        <v>200</v>
+      </c>
+      <c r="F13" s="41">
+        <v>200</v>
+      </c>
+      <c r="G13" s="41">
+        <v>200</v>
+      </c>
+      <c r="H13" s="41">
+        <v>200</v>
+      </c>
+      <c r="I13" s="41">
+        <v>200</v>
+      </c>
+      <c r="J13" s="41">
+        <v>200</v>
+      </c>
+      <c r="K13" s="41">
+        <v>200</v>
+      </c>
+      <c r="L13" s="41">
+        <v>200</v>
+      </c>
+      <c r="M13" s="41">
+        <v>200</v>
+      </c>
+      <c r="N13" s="41">
+        <v>200</v>
+      </c>
+      <c r="O13" s="41">
+        <v>200</v>
+      </c>
+      <c r="P13" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="41">
+        <v>0</v>
+      </c>
+      <c r="R13" s="41">
+        <v>0</v>
+      </c>
+      <c r="S13" s="41">
+        <v>0</v>
+      </c>
+      <c r="T13" s="41">
+        <v>0</v>
+      </c>
+      <c r="U13" s="41">
+        <v>0</v>
+      </c>
+      <c r="V13" s="41">
+        <v>0</v>
+      </c>
+      <c r="W13" s="41">
+        <v>0</v>
+      </c>
+      <c r="X13" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="D14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="E14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="F14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="G14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="H14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="I14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="J14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="K14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="L14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="M14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="N14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="O14" s="41">
+        <v>2000</v>
+      </c>
+      <c r="P14" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="41">
+        <v>0</v>
+      </c>
+      <c r="R14" s="41">
+        <v>0</v>
+      </c>
+      <c r="S14" s="41">
+        <v>0</v>
+      </c>
+      <c r="T14" s="41">
+        <v>0</v>
+      </c>
+      <c r="U14" s="41">
+        <v>0</v>
+      </c>
+      <c r="V14" s="41">
+        <v>0</v>
+      </c>
+      <c r="W14" s="41">
+        <v>0</v>
+      </c>
+      <c r="X14" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A15" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="D15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="E15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="F15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="G15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="H15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="I15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="J15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="K15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="L15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="M15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="N15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="O15" s="41">
+        <v>4000</v>
+      </c>
+      <c r="P15" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="41">
+        <v>0</v>
+      </c>
+      <c r="R15" s="41">
+        <v>0</v>
+      </c>
+      <c r="S15" s="41">
+        <v>0</v>
+      </c>
+      <c r="T15" s="41">
+        <v>0</v>
+      </c>
+      <c r="U15" s="41">
+        <v>0</v>
+      </c>
+      <c r="V15" s="41">
+        <v>0</v>
+      </c>
+      <c r="W15" s="41">
+        <v>0</v>
+      </c>
+      <c r="X15" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A16" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="D16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="E16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="F16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="G16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="H16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="I16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="J16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="K16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="L16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="M16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="N16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="O16" s="41">
+        <v>3000</v>
+      </c>
+      <c r="P16" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="41">
+        <v>0</v>
+      </c>
+      <c r="R16" s="41">
+        <v>0</v>
+      </c>
+      <c r="S16" s="41">
+        <v>0</v>
+      </c>
+      <c r="T16" s="41">
+        <v>0</v>
+      </c>
+      <c r="U16" s="41">
+        <v>0</v>
+      </c>
+      <c r="V16" s="41">
+        <v>0</v>
+      </c>
+      <c r="W16" s="41">
+        <v>0</v>
+      </c>
+      <c r="X16" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A17" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="41">
+        <v>1000</v>
+      </c>
+      <c r="D17" s="41">
+        <v>1000</v>
+      </c>
+      <c r="E17" s="41">
+        <v>1000</v>
+      </c>
+      <c r="F17" s="41">
+        <v>1000</v>
+      </c>
+      <c r="G17" s="41">
+        <v>1000</v>
+      </c>
+      <c r="H17" s="41">
+        <v>1000</v>
+      </c>
+      <c r="I17" s="41">
+        <v>1100</v>
+      </c>
+      <c r="J17" s="41">
+        <v>1100</v>
+      </c>
+      <c r="K17" s="41">
+        <v>1200</v>
+      </c>
+      <c r="L17" s="41">
+        <v>1200</v>
+      </c>
+      <c r="M17" s="41">
+        <v>1200</v>
+      </c>
+      <c r="N17" s="41">
+        <v>1300</v>
+      </c>
+      <c r="O17" s="41">
+        <v>1300</v>
+      </c>
+      <c r="P17" s="41">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="41">
+        <v>0</v>
+      </c>
+      <c r="R17" s="41">
+        <v>0</v>
+      </c>
+      <c r="S17" s="41">
+        <v>0</v>
+      </c>
+      <c r="T17" s="41">
+        <v>0</v>
+      </c>
+      <c r="U17" s="41">
+        <v>0</v>
+      </c>
+      <c r="V17" s="41">
+        <v>0</v>
+      </c>
+      <c r="W17" s="41">
+        <v>0</v>
+      </c>
+      <c r="X17" s="41">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="41">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="41">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="41">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changed Cash Ballance Card
</commit_message>
<xml_diff>
--- a/data/Сash_Flow_Budget.xlsx
+++ b/data/Сash_Flow_Budget.xlsx
@@ -1011,6 +1011,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Cash Flow Statement_Actual"/>
+      <sheetName val="Balance Sheet_Actual"/>
       <sheetName val="Sales_Actual"/>
       <sheetName val="COGS_Actual"/>
       <sheetName val="Working Capital_Actual"/>
@@ -1060,13 +1061,14 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>

</xml_diff>